<commit_message>
Refactor primary VPT chain and regenerate full outputs/methodology
</commit_message>
<xml_diff>
--- a/outputs/model_discounts/model_discounts_output.xlsx
+++ b/outputs/model_discounts/model_discounts_output.xlsx
@@ -427,48 +427,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>standardized_type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n_obs</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>interpretation_note</t>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>logit</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Insufficient variation/data for occurrence model in current window.</t>
+          <t>No rows</t>
         </is>
       </c>
     </row>
@@ -483,48 +455,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>standardized_type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n_obs</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>interpretation_note</t>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ols_hc1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Insufficient discounted observations for depth model.</t>
+          <t>No rows</t>
         </is>
       </c>
     </row>
@@ -539,219 +483,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>standardized_type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n_obs</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>coef_EU_no_promo</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>coef_EU_with_promo</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>coef_Producer_no_promo</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>coef_Producer_with_promo</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>delta_EU</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>delta_Producer</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>promo_coef_present</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>promo_coef_depth</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>interpretation_note</t>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>butter</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1.535644521267677</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-1.660182202847171</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-3.999278302034052</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.766933115146946</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-3.195826724114848</v>
-      </c>
-      <c r="H2" t="n">
-        <v>5.766211417180998</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-0.8947798337292888</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Difference between no-promo and promo-controlled pass-through.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>cream</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>33</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1.543144113274722</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1.41819009958284</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-2.828347575510229</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-2.764913204007323</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-0.1249540136918827</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.06343437150290576</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-0.1271753750785895</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Difference between no-promo and promo-controlled pass-through.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hard_cheese</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>33</v>
-      </c>
-      <c r="C4" t="n">
-        <v>-1.566095507221104</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.1552460384676559</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.6140932156535026</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-0.8329859269793987</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.72134154568876</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-1.447079142632901</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-0.3639259312553088</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Difference between no-promo and promo-controlled pass-through.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>milk</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>33</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1.357731332296655</v>
-      </c>
-      <c r="D5" t="n">
-        <v>4.27157712515603</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-1.247354240050975</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-2.005255656927778</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2.913845792859375</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-0.7579014168768037</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-0.6067609497040047</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Difference between no-promo and promo-controlled pass-through.</t>
+          <t>No primary-chain silpo rows available to build discount comparison.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily primary-chain refactor, synthetic consumer module, updated outputs and methodology
</commit_message>
<xml_diff>
--- a/outputs/model_discounts/model_discounts_output.xlsx
+++ b/outputs/model_discounts/model_discounts_output.xlsx
@@ -427,20 +427,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>standardized_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>promo_signal</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>definition</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No rows</t>
+          <t>butter</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>butter</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cream</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cream</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>hard_cheese</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hard_cheese</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sour_cream</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sour_cream</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1 if |promo-controlled - observed| &gt; 0.02</t>
         </is>
       </c>
     </row>
@@ -455,20 +638,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>standardized_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>promo_depth_proxy</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>definition</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No rows</t>
+          <t>butter</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>butter</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cream</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cream</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>hard_cheese</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hard_cheese</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sour_cream</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sour_cream</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>absolute difference between promo-controlled and observed SR coefficients</t>
         </is>
       </c>
     </row>
@@ -483,12 +849,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>standardized_type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>model_family</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>coef_observed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>coef_promo_controlled</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>delta_promo_control</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -496,7 +892,372 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No primary-chain silpo rows available to build discount comparison.</t>
+          <t>butter</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ARDL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.2001943602714764</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2001943602714764</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>butter</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NARDL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.04860976737983126</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.04860976737983126</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cream</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ARDL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.02719087049912439</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.02719087049912439</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cream</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NARDL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.070469572016711</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.070469572016711</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>hard_cheese</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ARDL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1.045350879786881</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.045350879786881</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>hard_cheese</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NARDL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.03093538709143862</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.03093538709143862</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ECM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.03780420860354025</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.03780420860354025</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NARDL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1309588230301683</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1309588230301683</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ARDL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5.213950941002082</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.213950941002082</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NARDL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9816109260310832</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9816109260310832</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sour_cream</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ARDL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.09602698663315934</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.09602698663315934</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sour_cream</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NARDL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>prozorro_to_retail</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.02591699786459659</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-0.02591699786459659</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>positive delta means stronger transmission after promo control</t>
         </is>
       </c>
     </row>

</xml_diff>